<commit_message>
Refactor data processing scripts and update datasets
Renamed and reorganized R scripts for data transformation, overview, and appendix generation. Enhanced data processing in 1_a_data_trans.R to improve monthly and yearly data handling, including reconstruction and consistency checks. Updated multiple Excel and image files in Data and Outcome directories, and regenerated month.RData to reflect these changes.
</commit_message>
<xml_diff>
--- a/Data/Population/1992-2023.xlsx
+++ b/Data/Population/1992-2023.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2024/13 NIDS TH/Code/Data/Population/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="356" documentId="11_AD4DA82427541F7ACA7EB83DB8CE2D986AE8DE17" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{303A4394-B27B-4EC2-9F43-8BB82DC60BF8}"/>
+  <xr:revisionPtr revIDLastSave="367" documentId="11_AD4DA82427541F7ACA7EB83DB8CE2D986AE8DE17" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D73E3A44-5247-4BE2-B5F9-0D37633729C1}"/>
   <bookViews>
-    <workbookView xWindow="4040" yWindow="1590" windowWidth="32600" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3380" yWindow="3380" windowWidth="28800" windowHeight="15460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="2" r:id="rId1"/>
     <sheet name="age" sheetId="1" r:id="rId2"/>
     <sheet name="province" sheetId="4" r:id="rId3"/>
     <sheet name="age_un" sheetId="3" r:id="rId4"/>
+    <sheet name="wpp" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="115">
   <si>
     <t>YEAR</t>
   </si>
@@ -8353,4 +8354,314 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EE4E79E-0A94-429F-BFB4-FC994A6A2D3A}">
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="12.58203125" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1990</v>
+      </c>
+      <c r="B2" s="3">
+        <v>54738329</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1991</v>
+      </c>
+      <c r="B3" s="3">
+        <v>55637434</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1992</v>
+      </c>
+      <c r="B4" s="3">
+        <v>56528834.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1993</v>
+      </c>
+      <c r="B5" s="3">
+        <v>57408198.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1994</v>
+      </c>
+      <c r="B6" s="3">
+        <v>58260854</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1995</v>
+      </c>
+      <c r="B7" s="3">
+        <v>59098232.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1996</v>
+      </c>
+      <c r="B8" s="3">
+        <v>59920064</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1997</v>
+      </c>
+      <c r="B9" s="3">
+        <v>60724584.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1998</v>
+      </c>
+      <c r="B10" s="3">
+        <v>61522630.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1999</v>
+      </c>
+      <c r="B11" s="3">
+        <v>62299043.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2000</v>
+      </c>
+      <c r="B12" s="3">
+        <v>63007815</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2001</v>
+      </c>
+      <c r="B13" s="3">
+        <v>63651141.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2002</v>
+      </c>
+      <c r="B14" s="3">
+        <v>64266436.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2003</v>
+      </c>
+      <c r="B15" s="3">
+        <v>64868166.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2004</v>
+      </c>
+      <c r="B16" s="3">
+        <v>65452047</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2005</v>
+      </c>
+      <c r="B17" s="3">
+        <v>66017419.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2006</v>
+      </c>
+      <c r="B18" s="3">
+        <v>66567687</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2007</v>
+      </c>
+      <c r="B19" s="3">
+        <v>67102394.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2008</v>
+      </c>
+      <c r="B20" s="3">
+        <v>67619830.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2009</v>
+      </c>
+      <c r="B21" s="3">
+        <v>68121080</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2010</v>
+      </c>
+      <c r="B22" s="3">
+        <v>68579447.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2011</v>
+      </c>
+      <c r="B23" s="3">
+        <v>69007208</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2012</v>
+      </c>
+      <c r="B24" s="3">
+        <v>69436098</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2013</v>
+      </c>
+      <c r="B25" s="3">
+        <v>69845114.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2014</v>
+      </c>
+      <c r="B26" s="3">
+        <v>70216366.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2015</v>
+      </c>
+      <c r="B27" s="3">
+        <v>70540795.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2016</v>
+      </c>
+      <c r="B28" s="3">
+        <v>70859841.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>2017</v>
+      </c>
+      <c r="B29" s="3">
+        <v>71160187</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>2018</v>
+      </c>
+      <c r="B30" s="3">
+        <v>71376078.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>2019</v>
+      </c>
+      <c r="B31" s="3">
+        <v>71522271</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2020</v>
+      </c>
+      <c r="B32" s="3">
+        <v>71641483.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>2021</v>
+      </c>
+      <c r="B33" s="3">
+        <v>71727332</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2022</v>
+      </c>
+      <c r="B34" s="3">
+        <v>71735329</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>2023</v>
+      </c>
+      <c r="B35" s="3">
+        <v>71702435</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>2024</v>
+      </c>
+      <c r="B36" s="3">
+        <v>71668011</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>2025</v>
+      </c>
+      <c r="B37" s="3">
+        <v>71619863</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update incidence/mortality rates and regional data processing
Changed incidence and mortality calculations from per 10 million to per 100,000 population in multiple scripts. Enhanced regional data processing in 4_a_province.R to include new data sources, population handling, and location name normalization. Updated output image dimensions and file paths, and added new data file for figure 6.
</commit_message>
<xml_diff>
--- a/Data/Population/1992-2023.xlsx
+++ b/Data/Population/1992-2023.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2024/13 NIDS TH/Code/Data/Population/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2024/13 NIDS TH/ID_TH/Data/Population/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="367" documentId="11_AD4DA82427541F7ACA7EB83DB8CE2D986AE8DE17" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D73E3A44-5247-4BE2-B5F9-0D37633729C1}"/>
   <bookViews>
-    <workbookView xWindow="3380" yWindow="3380" windowWidth="28800" windowHeight="15460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="28800" windowHeight="15460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="2" r:id="rId1"/>

</xml_diff>